<commit_message>
IVT, ABP Demo, EmailTextToPay QA2 changes
</commit_message>
<xml_diff>
--- a/KatalonData/ABPTestData/PaymentsACH.xlsx
+++ b/KatalonData/ABPTestData/PaymentsACH.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2179" uniqueCount="474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2187" uniqueCount="478">
   <si>
     <t>Result</t>
   </si>
@@ -1737,6 +1737,18 @@
   </si>
   <si>
     <t>Fri Sep 25 20:34:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Oct 08 01:42:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Oct 08 01:43:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Oct 08 01:44:09 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Oct 08 01:45:04 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -4071,10 +4083,10 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>436</v>
+        <v>477</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="1" t="s">

</xml_diff>